<commit_message>
Arm 2 (D10): use measured 18.5cm corner distance, 9.51 us/deg
Refit of the 2026-09-29 sweep with the measured shaft-to-corner distance
(was an assumed 18cm): 9.51 us/deg, centre unchanged at 1350us, worst
point 1.4 deg off the straight line.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JWjsACi7yRDojxi7bsVa7w
</commit_message>
<xml_diff>
--- a/engr489-firmware/tools/servo_sweep/servo2_angles.xlsx
+++ b/engr489-firmware/tools/servo_sweep/servo2_angles.xlsx
@@ -201,7 +201,7 @@
   <commentList>
     <comment ref="E4" authorId="0" shapeId="0">
       <text>
-        <t>ASSUMED: bicep joint-to-joint length (L_UP = 180 mm). Measure it and replace this.</t>
+        <t>Measured by you: 18.5 cm shaft centre to the measured corner.</t>
       </text>
     </comment>
     <comment ref="E5" authorId="0" shapeId="0">
@@ -558,11 +558,11 @@
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>18</v>
+        <v>18.5</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>ASSUMED: bicep joint-to-joint length (L_UP = 180 mm). Measure it and replace this.</t>
+          <t>Measured by you: 18.5 cm shaft centre to the measured corner.</t>
         </is>
       </c>
     </row>

</xml_diff>